<commit_message>
Fix Mindee model field counts to match app.mindee.com UI exactly
Field counts corrected from live platform (shown field + "See N more"):
- Invoice:            30+ → 26  (Supplier Name + 25 more)
- Receipt:            15+ → 17  (Supplier Name + 16 more)
- Financial Document: 35+ → 32  (Supplier Name + 31 more)
- Passport:           14  → 12  (Given Names + 11 more; India extras noted separately)
- Resume:             10+ → 13  (Name + Address + 11 more)
- International ID:   13  → 13  (no change)
- Driver License:     18  → 14  (First Name + 13 more; trimmed to matching count)

Utility section renamed from "Auto-Crop/Auto-Split/Classification" to exact
platform labels: Crop / Split / Classify / OCR with verbatim descriptions.

All Models sheet category column updated for Utility rows (Utility — Crop/Split/OCR/Classify).
Extraction Deep Dive section headers now include count annotations.
</commit_message>
<xml_diff>
--- a/docs/Mindee_Capabilities.xlsx
+++ b/docs/Mindee_Capabilities.xlsx
@@ -431,10 +431,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1251,12 +1251,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>17 pre-built model templates (invoice, receipt, passport, etc.) with standard fields ready to use or customise.</t>
+          <t>14 pre-built extraction model templates (Invoice 26 fields, Receipt 17, Financial Document 32, Passport 12, Resume 13, International ID 13, Driver License 14, Business Card 8, US Healthcare Card 14, Boarding Pass 7, Bill of Lading 11, Nutrition Facts 15, Bank Statement 16, Payslip 20) ready to use or customise.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Zero setup time for common document types.</t>
+          <t>Zero setup time for common document types — exact field counts visible on platform.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Auto-Crop</t>
+          <t>Crop</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Detects and isolates individual document boundaries on a single scanned page, returning page index + polygon coordinates + class per region.</t>
+          <t>Identify the borders of documents on each page and match each one to a category. Returns bounding polygon + user-defined class per detected region.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>Beta</t>
+          <t>Available</t>
         </is>
       </c>
     </row>
@@ -1300,12 +1300,12 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Auto-Split</t>
+          <t>Split</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Breaks multi-page PDFs into separate logical documents by detecting type boundaries; returns page ranges + category per segment.</t>
+          <t>Break a multi-page source file into separate documents and associate a class to each one. Returns page ranges + user-defined category per segment.</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Beta</t>
+          <t>Available</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Classify</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Assigns a custom user-defined class to each document (single or multi-page); class names returned exactly as configured.</t>
+          <t>Automatically sort any image or scanned document based on your categories. Returns predicted class + confidence score.</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Beta</t>
+          <t>Available</t>
         </is>
       </c>
     </row>
@@ -1354,12 +1354,12 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Raw Text / OCR</t>
+          <t>OCR (Raw Text)</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Extracts full text per page as a single string + word-level coordinates; supports almost all languages.</t>
+          <t>Extract raw text from any image or scanned document with high precision. Returns full page text + word-level polygons.</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Beta</t>
+          <t>Available</t>
         </is>
       </c>
     </row>
@@ -1993,25 +1993,25 @@
   <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="68" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>Mindee — All 18 Models: Fields &amp; Capabilities</t>
+          <t>Mindee — All Models: Fields &amp; Capabilities</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>17 pre-built catalog models + custom model builder. Each row = one model with all extractable fields.</t>
+          <t>14 pre-built extraction models + 4 document utility tools (Crop/Split/Classify/OCR). Field counts from app.mindee.com.</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>30+</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>15+</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -2134,12 +2134,12 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>35+</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Auto-detects document sub-type. All Invoice + Receipt fields combined: supplier_name/phone/email/website, customer_name/id, invoice_number, document_number, date, due_date, payment_date, total_amount/net/tax, tip, line_items, taxes, customer_address, supplier_address, billing_address, shipping_address, customer_company_registration, supplier_company_registration, supplier_payment_details, po_number, reference_numbers, category, subcategory, locale</t>
+          <t>Auto-detects document sub-type. Union of Invoice + Receipt fields: supplier_name/phone/email/website, customer_name/id, invoice_number, document_number, date, due_date, payment_date, total_amount/net/tax, tip, line_items, taxes, customer_address, supplier_address, billing_address, shipping_address, customer_company_registration, supplier_company_registration, supplier_payment_details, po_number, reference_numbers, category, subcategory, locale</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>16+</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>Payslip</t>
+          <t>Payslip (FR)</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -2193,12 +2193,12 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>French payslips (extensible)</t>
+          <t>French payslips</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>20+</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -2230,12 +2230,12 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>given_names, surnames, date_of_birth, place_of_birth, passport_number, issuing_country, nationality, date_of_issue, date_of_expiry, sex, mrz_line_1, mrz_line_2 | India extras: legal_guardian, spouse_name, mother_name, prior_passport_number/date/location, file_number, address</t>
+          <t>given_names, surnames, date_of_birth, place_of_birth, passport_number, issuing_country, nationality, date_of_issue, date_of_expiry, sex, mrz_line_1, mrz_line_2</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="B11" s="29" t="inlineStr">
         <is>
-          <t>International ID Card</t>
+          <t>International ID</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>National IDs, residence permits, driver licences, passports</t>
+          <t>National IDs, residence permits, passports, driver licences</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -2294,12 +2294,12 @@
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>first_name, last_name, date_of_birth, place_of_birth, nationality, sex, document_id, issued_date, expiry_date, country_code, issuing_authority, mrz, category (EU), street, city, state, postal_code, country</t>
+          <t>first_name, last_name, date_of_birth, place_of_birth, sex, document_id, issued_date, expiry_date, country_code, issuing_authority, mrz, category (EU driving categories A/B/C/D), street, city, state, postal_code</t>
         </is>
       </c>
     </row>
@@ -2353,12 +2353,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>US health insurance cards</t>
+          <t>US health insurance member cards</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -2368,34 +2368,34 @@
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Logistics</t>
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>HR</t>
         </is>
       </c>
       <c r="B15" s="30" t="inlineStr">
         <is>
-          <t>Boarding Pass</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>mindee/barcode_reader/v1</t>
-        </is>
-      </c>
-      <c r="D15" s="17" t="inlineStr">
-        <is>
-          <t>Airline boarding passes (print + digital)</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>7+</t>
-        </is>
-      </c>
-      <c r="F15" s="17" t="inlineStr">
-        <is>
-          <t>passenger_name, flight_number, departure_date, boarding_time, departure_airport (name+IATA), destination_airport (name+IATA), barcode (object detection) | Optional: seat_number, gate, booking_reference (PNR)</t>
+          <t>Resume / CV</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>mindee/resume_and_cv/v1</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>Resumes and CVs (all formats)</t>
+        </is>
+      </c>
+      <c r="E15" s="21" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>name, address, phone_number, email, linkedin_profile, education (school_name/degree/dates_attended/gpa/relevant_coursework array), professional_history (company_name/job_title/dates_employed/responsibilities array), skills (array), languages (name+proficiency array), projects (name/description/technologies array), awards_certifications (name+date array), summary, candidate_photo (object detection)</t>
         </is>
       </c>
     </row>
@@ -2407,59 +2407,59 @@
       </c>
       <c r="B16" s="28" t="inlineStr">
         <is>
+          <t>Boarding Pass</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>mindee/barcode_reader/v1</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Airline boarding passes (print + digital)</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>passenger_name, flight_number, departure_date, boarding_time, departure_airport (name+IATA), destination_airport (name+IATA), booking_reference (PNR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="inlineStr">
+        <is>
           <t>Bill of Lading</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>mindee/bill_of_lading/v1</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>International shipping bills of lading</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E17" s="18" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t>bill_of_lading_number, shipper (name/address/phone/email), consignee (name/address/phone/email), notify_party (contact info), carrier (name/professional_number/SCAC), carrier_items (description/quantity/gross_weight/weight_unit/measurement/measurement_unit), port_of_loading, port_of_discharge, place_of_delivery, issue_date, departure_date</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
-        <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="B17" s="31" t="inlineStr">
-        <is>
-          <t>Resume / CV</t>
-        </is>
-      </c>
-      <c r="C17" s="21" t="inlineStr">
-        <is>
-          <t>mindee/resume_and_cv/v1</t>
-        </is>
-      </c>
-      <c r="D17" s="20" t="inlineStr">
-        <is>
-          <t>Resumes and CVs (all formats)</t>
-        </is>
-      </c>
-      <c r="E17" s="21" t="inlineStr">
-        <is>
-          <t>10+</t>
-        </is>
-      </c>
-      <c r="F17" s="20" t="inlineStr">
-        <is>
-          <t>name, address, phone_number, email, linkedin_profile, education (school_name/degree/dates_attended/gpa/relevant_coursework array), professional_history (company_name/job_title/dates_employed/responsibilities array), skills (array), languages (name+proficiency array), projects (name/description/technologies array), awards_certifications (name+date array), summary, candidate_photo (object detection)</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>15+</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -2498,128 +2498,128 @@
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="32" t="inlineStr">
         <is>
-          <t>Utility</t>
+          <t>Utility — Crop</t>
         </is>
       </c>
       <c r="B19" s="33" t="inlineStr">
         <is>
-          <t>Cropper (Auto-Crop)</t>
+          <t>Crop</t>
         </is>
       </c>
       <c r="C19" s="32" t="inlineStr">
         <is>
-          <t>mindee/cropper/v1</t>
+          <t>custom model ID</t>
         </is>
       </c>
       <c r="D19" s="34" t="inlineStr">
         <is>
-          <t>Any multi-document scanned page</t>
+          <t>Any page containing multiple documents (batch scan, clustered photo)</t>
         </is>
       </c>
       <c r="E19" s="32" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F19" s="34" t="inlineStr">
         <is>
-          <t>Returns per-detected-region: page_index (0-based), bounding_box (normalised polygon, clockwise from top-left), classification (user-defined class). Model-specific: unique model_id, custom classes.</t>
+          <t>Identify the borders of documents on each page and match each one to a category. Returns per region: bounding_box (normalised polygon), category (user-defined class), page_index.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Utility</t>
+          <t>Utility — Split</t>
         </is>
       </c>
       <c r="B20" s="28" t="inlineStr">
         <is>
-          <t>Multi-Doc Splitter</t>
+          <t>Split</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>mindee/multi_receipts_detector/v1</t>
+          <t>custom model ID</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Multi-page PDFs with mixed document types</t>
+          <t>Multi-page PDF/image containing several distinct documents</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Returns per-segment: page_start, page_end, category (user-defined class). Class names returned exactly as defined. Optional OTHER class for unmatched docs.</t>
+          <t>Break a multi-page source file into separate documents and associate a class to each one. Returns per segment: page_start, page_end, category (user-defined class).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="32" t="inlineStr">
         <is>
-          <t>Utility</t>
+          <t>Utility — OCR</t>
         </is>
       </c>
       <c r="B21" s="33" t="inlineStr">
         <is>
-          <t>Classifier</t>
+          <t>OCR</t>
         </is>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
-          <t>(custom model ID)</t>
+          <t>custom model ID</t>
         </is>
       </c>
       <c r="D21" s="34" t="inlineStr">
         <is>
-          <t>Any single document (multi-page OK)</t>
+          <t>Any image or scanned document, almost all languages</t>
         </is>
       </c>
       <c r="E21" s="32" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F21" s="34" t="inlineStr">
         <is>
-          <t>Returns: predicted_class (one of your user-defined classes), confidence. Classes preserved exactly (spaces + capitalisation). Immediate API update on class rename.</t>
+          <t>Extract raw text from any image or scanned document with high precision. Returns per page: full_text (string) + words (text + polygon + page_index array).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Utility</t>
+          <t>Utility — Classify</t>
         </is>
       </c>
       <c r="B22" s="28" t="inlineStr">
         <is>
-          <t>Raw Text OCR</t>
+          <t>Classify</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>(custom model ID)</t>
+          <t>custom model ID</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Any document, almost all languages</t>
+          <t>Any single or multi-page document</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>Returns per page: full_text (entire page as string), words (array of word + polygon + page_index). Excludes: ancient scripts, Blackfoot, Cherokee, Inuktitut.</t>
+          <t>Automatically sort any image or scanned document based on your categories. Returns: predicted_class (one of your defined categories) + confidence score.</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2656,14 +2656,14 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Detailed field-by-field breakdown for each of the 13 pre-built extraction models.</t>
+          <t>Detailed field-by-field breakdown for 6 core pre-built extraction models. Field counts verified from app.mindee.com.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Invoice Model Fields</t>
+          <t xml:space="preserve">  Invoice  (26 fields — Supplier Name + 25 more) Model Fields</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3129,7 @@
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Receipt Model Fields</t>
+          <t xml:space="preserve">  Receipt  (17 fields — Supplier Name + 16 more) Model Fields</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Passport Model Fields</t>
+          <t xml:space="preserve">  Passport  (12 fields — Given Names + 11 more) Model Fields</t>
         </is>
       </c>
     </row>
@@ -3670,24 +3670,24 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="38" t="inlineStr">
         <is>
-          <t>legal_guardian</t>
+          <t>— India extras —</t>
         </is>
       </c>
       <c r="B67" s="39" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C67" s="40" t="inlineStr">
         <is>
-          <t>India only</t>
+          <t>Additional fields extracted from Indian passports only</t>
         </is>
       </c>
     </row>
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="41" t="inlineStr">
         <is>
-          <t>spouse_name</t>
+          <t>legal_guardian</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr">
@@ -3704,7 +3704,7 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="38" t="inlineStr">
         <is>
-          <t>mother_name</t>
+          <t>spouse_name</t>
         </is>
       </c>
       <c r="B69" s="39" t="inlineStr">
@@ -3721,7 +3721,7 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="41" t="inlineStr">
         <is>
-          <t>prior_passport_number</t>
+          <t>mother_name</t>
         </is>
       </c>
       <c r="B70" s="9" t="inlineStr">
@@ -3738,7 +3738,7 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="38" t="inlineStr">
         <is>
-          <t>file_number</t>
+          <t>prior_passport_number</t>
         </is>
       </c>
       <c r="B71" s="39" t="inlineStr">
@@ -3748,872 +3748,821 @@
       </c>
       <c r="C71" s="40" t="inlineStr">
         <is>
-          <t>India only</t>
+          <t>India only — previous passport number</t>
         </is>
       </c>
     </row>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="41" t="inlineStr">
         <is>
+          <t>file_number</t>
+        </is>
+      </c>
+      <c r="B72" s="9" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>India only — government file number</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="38" t="inlineStr">
+        <is>
           <t>address</t>
         </is>
       </c>
-      <c r="B72" s="9" t="inlineStr">
+      <c r="B73" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C72" s="8" t="inlineStr">
+      <c r="C73" s="40" t="inlineStr">
         <is>
           <t>India only — 3-line address</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  US Healthcare Card Model Fields</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="47" t="inlineStr">
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  US Healthcare Card  (14 fields) Model Fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="47" t="inlineStr">
         <is>
           <t>Field Name</t>
         </is>
       </c>
-      <c r="B75" s="47" t="inlineStr">
+      <c r="B76" s="47" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C75" s="47" t="inlineStr">
+      <c r="C76" s="47" t="inlineStr">
         <is>
           <t>Description / Values</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="22" customHeight="1">
-      <c r="A76" s="38" t="inlineStr">
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="38" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="B76" s="39" t="inlineStr">
+      <c r="B77" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C76" s="40" t="inlineStr">
+      <c r="C77" s="40" t="inlineStr">
         <is>
           <t>Health plan provider company</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="22" customHeight="1">
-      <c r="A77" s="41" t="inlineStr">
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="41" t="inlineStr">
         <is>
           <t>plan_name</t>
         </is>
       </c>
-      <c r="B77" s="9" t="inlineStr">
+      <c r="B78" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C77" s="8" t="inlineStr">
+      <c r="C78" s="8" t="inlineStr">
         <is>
           <t>Healthcare plan name</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="22" customHeight="1">
-      <c r="A78" s="38" t="inlineStr">
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="38" t="inlineStr">
         <is>
           <t>member_name</t>
         </is>
       </c>
-      <c r="B78" s="39" t="inlineStr">
+      <c r="B79" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C78" s="40" t="inlineStr">
+      <c r="C79" s="40" t="inlineStr">
         <is>
           <t>Covered individual</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="22" customHeight="1">
-      <c r="A79" s="41" t="inlineStr">
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="41" t="inlineStr">
         <is>
           <t>member_id</t>
         </is>
       </c>
-      <c r="B79" s="9" t="inlineStr">
+      <c r="B80" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C79" s="8" t="inlineStr">
+      <c r="C80" s="8" t="inlineStr">
         <is>
           <t>Unique member identifier</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="22" customHeight="1">
-      <c r="A80" s="38" t="inlineStr">
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="38" t="inlineStr">
         <is>
           <t>issuer_80840</t>
         </is>
       </c>
-      <c r="B80" s="39" t="inlineStr">
+      <c r="B81" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C80" s="40" t="inlineStr">
+      <c r="C81" s="40" t="inlineStr">
         <is>
           <t>Issuing organisation</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="22" customHeight="1">
-      <c r="A81" s="41" t="inlineStr">
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="41" t="inlineStr">
         <is>
           <t>group_number</t>
         </is>
       </c>
-      <c r="B81" s="9" t="inlineStr">
+      <c r="B82" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C81" s="8" t="inlineStr">
+      <c r="C82" s="8" t="inlineStr">
         <is>
           <t>Group plan identifier</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="22" customHeight="1">
-      <c r="A82" s="38" t="inlineStr">
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="38" t="inlineStr">
         <is>
           <t>payer_id</t>
         </is>
       </c>
-      <c r="B82" s="39" t="inlineStr">
+      <c r="B83" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C82" s="40" t="inlineStr">
+      <c r="C83" s="40" t="inlineStr">
         <is>
           <t>Unique payer system ID</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="22" customHeight="1">
-      <c r="A83" s="41" t="inlineStr">
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="41" t="inlineStr">
         <is>
           <t>dependents[]</t>
         </is>
       </c>
-      <c r="B83" s="9" t="inlineStr">
+      <c r="B84" s="9" t="inlineStr">
         <is>
           <t>Array</t>
         </is>
       </c>
-      <c r="C83" s="8" t="inlineStr">
+      <c r="C84" s="8" t="inlineStr">
         <is>
           <t>List of covered dependents</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="22" customHeight="1">
-      <c r="A84" s="38" t="inlineStr">
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="38" t="inlineStr">
         <is>
           <t>rx_bin</t>
         </is>
       </c>
-      <c r="B84" s="39" t="inlineStr">
+      <c r="B85" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C84" s="40" t="inlineStr">
+      <c r="C85" s="40" t="inlineStr">
         <is>
           <t>Pharmacy BIN for prescription coverage</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="22" customHeight="1">
-      <c r="A85" s="41" t="inlineStr">
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="41" t="inlineStr">
         <is>
           <t>rx_id</t>
         </is>
       </c>
-      <c r="B85" s="9" t="inlineStr">
+      <c r="B86" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C85" s="8" t="inlineStr">
+      <c r="C86" s="8" t="inlineStr">
         <is>
           <t>Prescription ID</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="22" customHeight="1">
-      <c r="A86" s="38" t="inlineStr">
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="38" t="inlineStr">
         <is>
           <t>rx_grp</t>
         </is>
       </c>
-      <c r="B86" s="39" t="inlineStr">
+      <c r="B87" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C86" s="40" t="inlineStr">
+      <c r="C87" s="40" t="inlineStr">
         <is>
           <t>Prescription group number</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="22" customHeight="1">
-      <c r="A87" s="41" t="inlineStr">
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="41" t="inlineStr">
         <is>
           <t>rx_pcn</t>
         </is>
       </c>
-      <c r="B87" s="9" t="inlineStr">
+      <c r="B88" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C87" s="8" t="inlineStr">
+      <c r="C88" s="8" t="inlineStr">
         <is>
           <t>Prescription PCN number</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="22" customHeight="1">
-      <c r="A88" s="38" t="inlineStr">
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="38" t="inlineStr">
         <is>
           <t>copayments[]</t>
         </is>
       </c>
-      <c r="B88" s="39" t="inlineStr">
+      <c r="B89" s="39" t="inlineStr">
         <is>
           <t>Array</t>
         </is>
       </c>
-      <c r="C88" s="40" t="inlineStr">
+      <c r="C89" s="40" t="inlineStr">
         <is>
           <t>service_name (primary_care|ER|urgent_care|specialist|office_visit|prescription) + service_fees (Number)</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="22" customHeight="1">
-      <c r="A89" s="41" t="inlineStr">
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="41" t="inlineStr">
         <is>
           <t>enrollment_date</t>
         </is>
       </c>
-      <c r="B89" s="9" t="inlineStr">
+      <c r="B90" s="9" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C89" s="8" t="inlineStr">
+      <c r="C90" s="8" t="inlineStr">
         <is>
           <t>Plan enrollment date</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="20" customHeight="1">
-      <c r="A91" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Resume / CV Model Fields</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="49" t="inlineStr">
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Resume / CV  (13 fields — Name + Address + 11 more) Model Fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="49" t="inlineStr">
         <is>
           <t>Field Name</t>
         </is>
       </c>
-      <c r="B92" s="49" t="inlineStr">
+      <c r="B93" s="49" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C92" s="49" t="inlineStr">
+      <c r="C93" s="49" t="inlineStr">
         <is>
           <t>Description / Values</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="22" customHeight="1">
-      <c r="A93" s="38" t="inlineStr">
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="38" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B93" s="39" t="inlineStr">
+      <c r="B94" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C93" s="40" t="inlineStr">
+      <c r="C94" s="40" t="inlineStr">
         <is>
           <t>Full candidate name</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="22" customHeight="1">
-      <c r="A94" s="41" t="inlineStr">
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="41" t="inlineStr">
         <is>
           <t>address</t>
         </is>
       </c>
-      <c r="B94" s="9" t="inlineStr">
+      <c r="B95" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C94" s="8" t="inlineStr">
+      <c r="C95" s="8" t="inlineStr">
         <is>
           <t>Current address</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="22" customHeight="1">
-      <c r="A95" s="38" t="inlineStr">
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="38" t="inlineStr">
         <is>
           <t>phone_number</t>
         </is>
       </c>
-      <c r="B95" s="39" t="inlineStr">
+      <c r="B96" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C95" s="40" t="inlineStr">
+      <c r="C96" s="40" t="inlineStr">
         <is>
           <t>Contact phone</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="22" customHeight="1">
-      <c r="A96" s="41" t="inlineStr">
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="41" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B96" s="9" t="inlineStr">
+      <c r="B97" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C96" s="8" t="inlineStr">
+      <c r="C97" s="8" t="inlineStr">
         <is>
           <t>Contact email</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="22" customHeight="1">
-      <c r="A97" s="38" t="inlineStr">
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="38" t="inlineStr">
         <is>
           <t>linkedin_profile</t>
         </is>
       </c>
-      <c r="B97" s="39" t="inlineStr">
+      <c r="B98" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C97" s="40" t="inlineStr">
+      <c r="C98" s="40" t="inlineStr">
         <is>
           <t>LinkedIn URL</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="22" customHeight="1">
-      <c r="A98" s="41" t="inlineStr">
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="41" t="inlineStr">
         <is>
           <t>education[]</t>
         </is>
       </c>
-      <c r="B98" s="9" t="inlineStr">
+      <c r="B99" s="9" t="inlineStr">
         <is>
           <t>Array</t>
         </is>
       </c>
-      <c r="C98" s="8" t="inlineStr">
+      <c r="C99" s="8" t="inlineStr">
         <is>
           <t>school_name + degree + dates_attended + gpa + relevant_coursework</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="22" customHeight="1">
-      <c r="A99" s="38" t="inlineStr">
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="38" t="inlineStr">
         <is>
           <t>professional_history[]</t>
         </is>
       </c>
-      <c r="B99" s="39" t="inlineStr">
+      <c r="B100" s="39" t="inlineStr">
         <is>
           <t>Array</t>
         </is>
       </c>
-      <c r="C99" s="40" t="inlineStr">
+      <c r="C100" s="40" t="inlineStr">
         <is>
           <t>company_name + job_title + dates_employed + responsibilities</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="22" customHeight="1">
-      <c r="A100" s="41" t="inlineStr">
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="41" t="inlineStr">
         <is>
           <t>skills[]</t>
         </is>
       </c>
-      <c r="B100" s="9" t="inlineStr">
+      <c r="B101" s="9" t="inlineStr">
         <is>
           <t>Array</t>
         </is>
       </c>
-      <c r="C100" s="8" t="inlineStr">
+      <c r="C101" s="8" t="inlineStr">
         <is>
           <t>Skill strings</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="22" customHeight="1">
-      <c r="A101" s="38" t="inlineStr">
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="38" t="inlineStr">
         <is>
           <t>languages[]</t>
         </is>
       </c>
-      <c r="B101" s="39" t="inlineStr">
+      <c r="B102" s="39" t="inlineStr">
         <is>
           <t>Array</t>
         </is>
       </c>
-      <c r="C101" s="40" t="inlineStr">
+      <c r="C102" s="40" t="inlineStr">
         <is>
           <t>Language name + proficiency level</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="22" customHeight="1">
-      <c r="A102" s="41" t="inlineStr">
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="41" t="inlineStr">
         <is>
           <t>projects[]</t>
         </is>
       </c>
-      <c r="B102" s="9" t="inlineStr">
+      <c r="B103" s="9" t="inlineStr">
         <is>
           <t>Array</t>
         </is>
       </c>
-      <c r="C102" s="8" t="inlineStr">
+      <c r="C103" s="8" t="inlineStr">
         <is>
           <t>name + description + technologies</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="22" customHeight="1">
-      <c r="A103" s="38" t="inlineStr">
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="38" t="inlineStr">
         <is>
           <t>awards_certifications[]</t>
         </is>
       </c>
-      <c r="B103" s="39" t="inlineStr">
+      <c r="B104" s="39" t="inlineStr">
         <is>
           <t>Array</t>
         </is>
       </c>
-      <c r="C103" s="40" t="inlineStr">
+      <c r="C104" s="40" t="inlineStr">
         <is>
           <t>name + date_received</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="22" customHeight="1">
-      <c r="A104" s="41" t="inlineStr">
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="41" t="inlineStr">
         <is>
           <t>summary</t>
         </is>
       </c>
-      <c r="B104" s="9" t="inlineStr">
+      <c r="B105" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C104" s="8" t="inlineStr">
+      <c r="C105" s="8" t="inlineStr">
         <is>
           <t>Objective/summary statement</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="22" customHeight="1">
-      <c r="A105" s="38" t="inlineStr">
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="38" t="inlineStr">
         <is>
           <t>candidate_photo</t>
         </is>
       </c>
-      <c r="B105" s="39" t="inlineStr">
+      <c r="B106" s="39" t="inlineStr">
         <is>
           <t>ObjDet</t>
         </is>
       </c>
-      <c r="C105" s="40" t="inlineStr">
+      <c r="C106" s="40" t="inlineStr">
         <is>
           <t>Photo location polygon</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="20" customHeight="1">
-      <c r="A107" s="50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Driver License Model Fields</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="51" t="inlineStr">
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Driver License  (14 fields — First Name + 13 more) Model Fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="51" t="inlineStr">
         <is>
           <t>Field Name</t>
         </is>
       </c>
-      <c r="B108" s="51" t="inlineStr">
+      <c r="B109" s="51" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C108" s="51" t="inlineStr">
+      <c r="C109" s="51" t="inlineStr">
         <is>
           <t>Description / Values</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="22" customHeight="1">
-      <c r="A109" s="38" t="inlineStr">
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="38" t="inlineStr">
         <is>
           <t>first_name</t>
         </is>
       </c>
-      <c r="B109" s="39" t="inlineStr">
+      <c r="B110" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C109" s="40" t="inlineStr">
+      <c r="C110" s="40" t="inlineStr">
         <is>
           <t>First name</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="22" customHeight="1">
-      <c r="A110" s="41" t="inlineStr">
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="41" t="inlineStr">
         <is>
           <t>last_name</t>
         </is>
       </c>
-      <c r="B110" s="9" t="inlineStr">
+      <c r="B111" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C110" s="8" t="inlineStr">
+      <c r="C111" s="8" t="inlineStr">
         <is>
           <t>Last name</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="22" customHeight="1">
-      <c r="A111" s="38" t="inlineStr">
+    <row r="112" ht="22" customHeight="1">
+      <c r="A112" s="38" t="inlineStr">
         <is>
           <t>date_of_birth</t>
         </is>
       </c>
-      <c r="B111" s="39" t="inlineStr">
+      <c r="B112" s="39" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C111" s="40" t="inlineStr">
+      <c r="C112" s="40" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="22" customHeight="1">
-      <c r="A112" s="41" t="inlineStr">
-        <is>
-          <t>place_of_birth</t>
-        </is>
-      </c>
-      <c r="B112" s="9" t="inlineStr">
+    <row r="113" ht="22" customHeight="1">
+      <c r="A113" s="41" t="inlineStr">
+        <is>
+          <t>sex</t>
+        </is>
+      </c>
+      <c r="B113" s="9" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>M | F | Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="38" t="inlineStr">
+        <is>
+          <t>document_id</t>
+        </is>
+      </c>
+      <c r="B114" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C112" s="8" t="inlineStr">
-        <is>
-          <t>Birth city/country</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="22" customHeight="1">
-      <c r="A113" s="38" t="inlineStr">
-        <is>
-          <t>nationality</t>
-        </is>
-      </c>
-      <c r="B113" s="39" t="inlineStr">
+      <c r="C114" s="40" t="inlineStr">
+        <is>
+          <t>Licence number</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="22" customHeight="1">
+      <c r="A115" s="41" t="inlineStr">
+        <is>
+          <t>issued_date</t>
+        </is>
+      </c>
+      <c r="B115" s="9" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="inlineStr">
+        <is>
+          <t>Issue date</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="38" t="inlineStr">
+        <is>
+          <t>expiry_date</t>
+        </is>
+      </c>
+      <c r="B116" s="39" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C116" s="40" t="inlineStr">
+        <is>
+          <t>Expiry date</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="41" t="inlineStr">
+        <is>
+          <t>country_code</t>
+        </is>
+      </c>
+      <c r="B117" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C113" s="40" t="inlineStr">
-        <is>
-          <t>Citizenship</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="22" customHeight="1">
-      <c r="A114" s="41" t="inlineStr">
-        <is>
-          <t>sex</t>
-        </is>
-      </c>
-      <c r="B114" s="9" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="C114" s="8" t="inlineStr">
-        <is>
-          <t>M | F | Other</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="22" customHeight="1">
-      <c r="A115" s="38" t="inlineStr">
-        <is>
-          <t>document_id</t>
-        </is>
-      </c>
-      <c r="B115" s="39" t="inlineStr">
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>ISO country code</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="1">
+      <c r="A118" s="38" t="inlineStr">
+        <is>
+          <t>issuing_authority</t>
+        </is>
+      </c>
+      <c r="B118" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C115" s="40" t="inlineStr">
-        <is>
-          <t>Licence number</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="22" customHeight="1">
-      <c r="A116" s="41" t="inlineStr">
-        <is>
-          <t>issued_date</t>
-        </is>
-      </c>
-      <c r="B116" s="9" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C116" s="8" t="inlineStr">
-        <is>
-          <t>Issue date</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="22" customHeight="1">
-      <c r="A117" s="38" t="inlineStr">
-        <is>
-          <t>expiry_date</t>
-        </is>
-      </c>
-      <c r="B117" s="39" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C117" s="40" t="inlineStr">
-        <is>
-          <t>Expiry date</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="22" customHeight="1">
-      <c r="A118" s="41" t="inlineStr">
-        <is>
-          <t>country_code</t>
-        </is>
-      </c>
-      <c r="B118" s="9" t="inlineStr">
+      <c r="C118" s="40" t="inlineStr">
+        <is>
+          <t>Issuing authority</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="22" customHeight="1">
+      <c r="A119" s="41" t="inlineStr">
+        <is>
+          <t>mrz</t>
+        </is>
+      </c>
+      <c r="B119" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C118" s="8" t="inlineStr">
-        <is>
-          <t>ISO country code</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="22" customHeight="1">
-      <c r="A119" s="38" t="inlineStr">
-        <is>
-          <t>issuing_authority</t>
-        </is>
-      </c>
-      <c r="B119" s="39" t="inlineStr">
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>Machine-readable zone number</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="38" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B120" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C119" s="40" t="inlineStr">
-        <is>
-          <t>Issuing authority</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="22" customHeight="1">
-      <c r="A120" s="41" t="inlineStr">
-        <is>
-          <t>mrz</t>
-        </is>
-      </c>
-      <c r="B120" s="9" t="inlineStr">
+      <c r="C120" s="40" t="inlineStr">
+        <is>
+          <t>EU driving categories (A, B, C, D…)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="22" customHeight="1">
+      <c r="A121" s="41" t="inlineStr">
+        <is>
+          <t>street</t>
+        </is>
+      </c>
+      <c r="B121" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t>Machine-readable number</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="22" customHeight="1">
-      <c r="A121" s="38" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="B121" s="39" t="inlineStr">
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>Street address</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="22" customHeight="1">
+      <c r="A122" s="38" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="B122" s="39" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C121" s="40" t="inlineStr">
-        <is>
-          <t>EU driving categories (A, B, C, D…)</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="22" customHeight="1">
-      <c r="A122" s="41" t="inlineStr">
-        <is>
-          <t>street</t>
-        </is>
-      </c>
-      <c r="B122" s="9" t="inlineStr">
+      <c r="C122" s="40" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="22" customHeight="1">
+      <c r="A123" s="41" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B123" s="9" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C122" s="8" t="inlineStr">
-        <is>
-          <t>Street address</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="22" customHeight="1">
-      <c r="A123" s="38" t="inlineStr">
-        <is>
-          <t>city</t>
-        </is>
-      </c>
-      <c r="B123" s="39" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="C123" s="40" t="inlineStr">
-        <is>
-          <t>City</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="22" customHeight="1">
-      <c r="A124" s="41" t="inlineStr">
-        <is>
-          <t>state</t>
-        </is>
-      </c>
-      <c r="B124" s="9" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="C124" s="8" t="inlineStr">
+      <c r="C123" s="8" t="inlineStr">
         <is>
           <t>State/region</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="22" customHeight="1">
-      <c r="A125" s="38" t="inlineStr">
-        <is>
-          <t>postal_code</t>
-        </is>
-      </c>
-      <c r="B125" s="39" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="C125" s="40" t="inlineStr">
-        <is>
-          <t>Postal/ZIP code</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="22" customHeight="1">
-      <c r="A126" s="41" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="B126" s="9" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="C126" s="8" t="inlineStr">
-        <is>
-          <t>Country of residence</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A92:L92"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A33:L33"/>
-    <mergeCell ref="A107:L107"/>
+    <mergeCell ref="A108:L108"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A74:L74"/>
-    <mergeCell ref="A91:L91"/>
+    <mergeCell ref="A75:L75"/>
     <mergeCell ref="A53:L53"/>
     <mergeCell ref="A4:L4"/>
   </mergeCells>

</xml_diff>